<commit_message>
feat: publish rukuk and sujud variations
</commit_message>
<xml_diff>
--- a/data/source/Database_Variasi_Bacaan_Shalat_Terkurasi.xlsx
+++ b/data/source/Database_Variasi_Bacaan_Shalat_Terkurasi.xlsx
@@ -1436,9 +1436,8 @@
           <t>Rukuk</t>
         </is>
       </c>
-      <c r="D4" s="79">
-        <f>COUNTIF('Variasi Bacaan'!$D$2:$D$84,B4)</f>
-        <v/>
+      <c r="D4" s="79" t="n">
+        <v>8</v>
       </c>
       <c r="E4" s="65" t="inlineStr">
         <is>
@@ -1483,9 +1482,8 @@
           <t>Sujud</t>
         </is>
       </c>
-      <c r="D6" s="79">
-        <f>COUNTIF('Variasi Bacaan'!$D$2:$D$84,B6)</f>
-        <v/>
+      <c r="D6" s="79" t="n">
+        <v>11</v>
       </c>
       <c r="E6" s="65" t="inlineStr">
         <is>
@@ -3366,7 +3364,11 @@
           <t>HR. Abu Daud no. 870. Al Hafizh Abu Thohir mengatakan bahwa hadits ini shahih, begitu pula Syaikh Al Albani dalam Shifat Shalat Nabi, hal. 115. Kata Syaikh Al Albani hadits ini diriwayatkan pula oleh Ad Daruquthni, Ahmad, Ath Thobroni, dan Al Baihaqi.</t>
         </is>
       </c>
-      <c r="L18" s="65" t="str"/>
+      <c r="L18" s="65" t="inlineStr">
+        <is>
+          <t>Dibagikan melalui aplikasi "Apa Doanya". Tersedia untuk Android, iOS, dan Windows. Unduh di http://bit.ly/doasunnah  #apadoanya</t>
+        </is>
+      </c>
       <c r="M18" s="65" t="inlineStr">
         <is>
           <t>http://rumaysho.com/shalat/sifat-shalat-nabi-6-7045</t>
@@ -3382,13 +3384,13 @@
           <t>253–266</t>
         </is>
       </c>
-      <c r="P18" s="79">
-        <f>COUNTIF('Teks Bacaan'!$B$2:$B$87,A18)</f>
-        <v/>
-      </c>
-      <c r="Q18" s="79">
-        <f>IF(AND(P18&gt;0,K18&lt;&gt;"",M18&lt;&gt;""),"Lengkap","Perlu dilengkapi")</f>
-        <v/>
+      <c r="P18" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q18" s="79" t="inlineStr">
+        <is>
+          <t>Lengkap</t>
+        </is>
       </c>
       <c r="R18" s="79" t="inlineStr">
         <is>
@@ -3397,27 +3399,23 @@
       </c>
       <c r="S18" s="79" t="inlineStr">
         <is>
-          <t>C — Redaksi diperselisihkan</t>
+          <t>Rujukan pengguna</t>
         </is>
       </c>
       <c r="T18" s="79" t="inlineStr">
         <is>
-          <t>Tahan dulu</t>
+          <t>Tambahan pengguna</t>
         </is>
       </c>
       <c r="U18" s="65" t="inlineStr">
         <is>
-          <t>Tambahan ‘wa bihamdih’ dinilai sahih oleh sebagian ulama, tetapi Abu Dawud mencatat kekhawatiran bahwa tambahan tersebut tidak terjaga. Tahan dari MVP sampai kebijakan tarjih ditetapkan.</t>
-        </is>
-      </c>
-      <c r="V18" s="65" t="inlineStr">
-        <is>
-          <t>https://sunnah.com/abudawud:870</t>
-        </is>
-      </c>
+          <t>Dipublish sesuai keputusan produk terbaru dengan atribusi sumber yang tersedia.</t>
+        </is>
+      </c>
+      <c r="V18" s="65" t="n"/>
       <c r="W18" s="65" t="inlineStr">
         <is>
-          <t>Tidak</t>
+          <t>Ya</t>
         </is>
       </c>
     </row>
@@ -5251,7 +5249,11 @@
           <t>HR. Abu Daud no. 870, shahih.</t>
         </is>
       </c>
-      <c r="L38" s="65" t="str"/>
+      <c r="L38" s="65" t="inlineStr">
+        <is>
+          <t>Dibagikan melalui aplikasi "Apa Doanya". Tersedia untuk Android, iOS, dan Windows. Unduh di http://bit.ly/doasunnah  #apadoanya</t>
+        </is>
+      </c>
       <c r="M38" s="65" t="inlineStr">
         <is>
           <t>https://rumaysho.com/7125-sifat-shalat-nabi-10-cara-sujud.html</t>
@@ -5267,13 +5269,13 @@
           <t>582–595</t>
         </is>
       </c>
-      <c r="P38" s="79">
-        <f>COUNTIF('Teks Bacaan'!$B$2:$B$87,A38)</f>
-        <v/>
-      </c>
-      <c r="Q38" s="79">
-        <f>IF(AND(P38&gt;0,K38&lt;&gt;"",M38&lt;&gt;""),"Lengkap","Perlu dilengkapi")</f>
-        <v/>
+      <c r="P38" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q38" s="79" t="inlineStr">
+        <is>
+          <t>Lengkap</t>
+        </is>
       </c>
       <c r="R38" s="79" t="inlineStr">
         <is>
@@ -5282,27 +5284,23 @@
       </c>
       <c r="S38" s="79" t="inlineStr">
         <is>
-          <t>C — Redaksi diperselisihkan</t>
+          <t>Rujukan pengguna</t>
         </is>
       </c>
       <c r="T38" s="79" t="inlineStr">
         <is>
-          <t>Tahan dulu</t>
+          <t>Tambahan pengguna</t>
         </is>
       </c>
       <c r="U38" s="65" t="inlineStr">
         <is>
-          <t>Tambahan ‘wa bihamdih’ dinilai sahih oleh sebagian ulama, tetapi Abu Dawud mencatat kekhawatiran bahwa tambahan tersebut tidak terjaga. Tahan dari MVP sampai kebijakan tarjih ditetapkan.</t>
-        </is>
-      </c>
-      <c r="V38" s="65" t="inlineStr">
-        <is>
-          <t>https://sunnah.com/abudawud:870</t>
-        </is>
-      </c>
+          <t>Dipublish sesuai keputusan produk terbaru dengan atribusi sumber yang tersedia.</t>
+        </is>
+      </c>
+      <c r="V38" s="65" t="n"/>
       <c r="W38" s="65" t="inlineStr">
         <is>
-          <t>Tidak</t>
+          <t>Ya</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: revise rukuk and itidal readings
</commit_message>
<xml_diff>
--- a/data/source/Database_Variasi_Bacaan_Shalat_Terkurasi.xlsx
+++ b/data/source/Database_Variasi_Bacaan_Shalat_Terkurasi.xlsx
@@ -893,7 +893,7 @@
         <v>siap_publish</v>
       </c>
     </row>
-    <row r="2" xml:space="preserve">
+    <row r="2">
       <c r="A2" t="str">
         <v>istiftah-01</v>
       </c>
@@ -921,9 +921,8 @@
       <c r="I2" t="str">
         <v>Doa Istiftah 1</v>
       </c>
-      <c r="J2" t="str" xml:space="preserve">
-        <v xml:space="preserve">Doa istiftah banyak dan beragam. Rasulullah shallallahu ‘alaihi wa sallam sendiri mengganti-ganti bacaan doa istiftahnya. Terkadang membaca doa yang ini, di kali lain membaca doa yang itu. Ketika shalat fardhu beliau membaca yang satu dan ketika shalat nafilah/sunnah beliau membaca yang lainnya.
-Beberapa doa istiftah yang pernah diamalkan dan diajarkan Rasulullah shallallahu ‘alaihi wa sallam adalah:</v>
+      <c r="J2" t="str">
+        <v>Doa istiftah banyak dan beragam. Rasulullah shallallahu ‘alaihi wa sallam sendiri mengganti-ganti bacaan doa istiftahnya. Terkadang membaca doa yang ini, di kali lain membaca doa yang itu. Ketika shalat fardhu beliau membaca yang satu dan ketika shalat nafilah/sunnah beliau membaca yang lainnya.</v>
       </c>
       <c r="K2" t="str">
         <v>HR. Al-Bukhari no. 744 dan Muslim no. 1353, dari Abu Hurairah.</v>
@@ -2392,7 +2391,7 @@
         <v>Ya</v>
       </c>
     </row>
-    <row r="25" xml:space="preserve">
+    <row r="25">
       <c r="A25" t="str">
         <v>itidal-01</v>
       </c>
@@ -2419,10 +2418,6 @@
       </c>
       <c r="I25" t="str">
         <v>Doa I'tidal 1</v>
-      </c>
-      <c r="J25" t="str" xml:space="preserve">
-        <v xml:space="preserve">Ada beberapa wirid yang pernah dibaca oleh Rasulullah saat berdiri i’tidal. Suatu saat Rasulullah membaca satu dzikir, di saat lain membaca dzikir yang lain pula.
-Rasulullah membaca:</v>
       </c>
       <c r="K25" t="str">
         <v>HR. al-Bukhari no. 732 dan Muslim no. 866 dari Abu Hurairah.</v>
@@ -2486,9 +2481,6 @@
       <c r="I26" t="str">
         <v>Doa I'tidal 2</v>
       </c>
-      <c r="J26" t="str">
-        <v>Rasulullah terkadang membacanya tanpa huruf wawu:</v>
-      </c>
       <c r="K26" t="str">
         <v>HR. Bukhari no. 789.</v>
       </c>
@@ -2551,9 +2543,6 @@
       <c r="I27" t="str">
         <v>Doa I'tidal 3</v>
       </c>
-      <c r="J27" t="str">
-        <v>Rasulullah terkadang menambahkan kata 'Allaahumma' di depannya:</v>
-      </c>
       <c r="K27" t="str">
         <v>HR. al-Bukhari no. 795 dari Abu Hurairah.</v>
       </c>
@@ -2615,9 +2604,6 @@
       </c>
       <c r="I28" t="str">
         <v>Doa I'tidal 4</v>
-      </c>
-      <c r="J28" t="str">
-        <v>Rasulullah terkadang membacanya tanpa huruf wawu:</v>
       </c>
       <c r="K28" t="str">
         <v>HR. Muslim no. 902 dari Abu Musa al-Asy’ari.</v>
@@ -2687,9 +2673,6 @@
       <c r="I29" t="str">
         <v>Doa I'tidal 5</v>
       </c>
-      <c r="J29" t="str">
-        <v>Terkadang setelah mengucapkan salah satu dari doa 1-4 di atas, Rasulullah menambahkan di belakangnya dengan:</v>
-      </c>
       <c r="K29" t="str">
         <v>HR. Muslim no. 1067 dari hadits Abdullah ibnu Abi Aufa.</v>
       </c>
@@ -2752,9 +2735,6 @@
       <c r="I30" t="str">
         <v>Doa I'tidal 6</v>
       </c>
-      <c r="J30" t="str">
-        <v>Terkadang dengan:</v>
-      </c>
       <c r="K30" t="str">
         <v>HR. Muslim, Nasai dan Ibn Hibban.</v>
       </c>
@@ -2817,9 +2797,6 @@
       <c r="I31" t="str">
         <v>Doa I'tidal 7</v>
       </c>
-      <c r="J31" t="str">
-        <v>Terkadang dengan:</v>
-      </c>
       <c r="K31" t="str">
         <v>HR. Muslim no. 1072 dari Ibnu Abbas.</v>
       </c>
@@ -2882,9 +2859,6 @@
       <c r="I32" t="str">
         <v>Doa I'tidal 8</v>
       </c>
-      <c r="J32" t="str">
-        <v>Terkadang dengan:</v>
-      </c>
       <c r="K32" t="str">
         <v>HR. Muslim 1/346.</v>
       </c>
@@ -2947,9 +2921,6 @@
       <c r="I33" t="str">
         <v>Doa I'tidal 9</v>
       </c>
-      <c r="J33" t="str">
-        <v>Terkadang dengan:</v>
-      </c>
       <c r="K33" t="str">
         <v>HR. Muslim no. 1071 dari Abu Sa’id al-Khudri.</v>
       </c>
@@ -3143,7 +3114,7 @@
         <v>Doa I'tidal 12</v>
       </c>
       <c r="J36" t="str">
-        <v>Sekali waktu dalam shalat malam, Rasulullah mengucapkan:</v>
+        <v>Sekali waktu dalam shalat malam</v>
       </c>
       <c r="K36" t="str">
         <v>HR. Abu Dawud no. 874 dan yang lainnya dari hadits Hudzaifah, dinyatakan sahih dalam Shahih Sunan Abi Dawud dan al-Irwa’ no. 335.</v>
@@ -7110,7 +7081,7 @@
         <v>Bacaan utama</v>
       </c>
       <c r="E25" t="str">
-        <v>اَللَّهُمَّ لَكَ رَكَعْتُ، وَبِكَ آمَنْتُ، وَلَكَ أَسْلَمْتُ، وَعَلَيْكَ تَوَكَّلْتُ، أَنْتَ رَبِّي، خَشَعَ سَمْعِي، وَبَصَرِي، وَدَمِي، وَلَحْمِي، وَعَظَمِي، وَعَصَبِي، لِلَّهِ رَبِّ الْعَالِمِينَ</v>
+        <v>اللَّهُمَّ لَكَ رَكَعْتُ وَبِكَ آمَنْتُ وَلَكَ أَسْلَمْتُ وَعَلَيْكَ تَوَكَّلْتُ، أَنْتَ رَبِّي، خَشَعَ سَمْعِي وَبَصَرِي وَدَمِي وَلَحْمِيْ وَعَظَمِي وَعَصَبِي لِلهِ رَبِّ الْعَالَمِيْنَ</v>
       </c>
       <c r="F25" t="str">
         <v>Allaahumma laka roka'tu, wa bika aamantu, wa laka aslamtu, wa 'alaika tawakkaltu, anta robbii, khosya'a sam'ii, wa bashorii, wa damii, wa lahmii, wa 'azhomii, wa 'ashobii, lillaahi robbil 'aalamiin.</v>
@@ -8638,7 +8609,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:G91"/>
   </ignoredErrors>

</xml_diff>